<commit_message>
Remove puzzle pages for keywords 2 and 3
</commit_message>
<xml_diff>
--- a/imports/20261005-002.xlsx
+++ b/imports/20261005-002.xlsx
@@ -1223,108 +1223,112 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="3" outlineLevelCol="6"/>
-  <cols>
-    <col min="1" max="1" width="11.2115384615385" customWidth="1"/>
-    <col min="3" max="3" width="13.2980769230769" customWidth="1"/>
-    <col min="4" max="4" width="22.4326923076923" customWidth="1"/>
-    <col min="5" max="5" width="28.2019230769231" customWidth="1"/>
-    <col min="6" max="6" width="20.1923076923077" customWidth="1"/>
-    <col min="7" max="7" width="22.1153846153846" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4"/>
-      <c r="F4">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr/>
+  <ns0:dimension ref="A1:G4"/>
+  <ns0:sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="3" outlineLevelCol="6"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="11.2115384615385" customWidth="1"/>
+    <ns0:col min="3" max="3" width="13.2980769230769" customWidth="1"/>
+    <ns0:col min="4" max="4" width="22.4326923076923" customWidth="1"/>
+    <ns0:col min="5" max="5" width="28.2019230769231" customWidth="1"/>
+    <ns0:col min="6" max="6" width="20.1923076923077" customWidth="1"/>
+    <ns0:col min="7" max="7" width="22.1153846153846" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:7">
+      <ns0:c r="A1" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="D1" t="s">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="E1" t="s">
+        <ns0:v>4</ns0:v>
+      </ns0:c>
+      <ns0:c r="F1" t="s">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="G1" t="s">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:7">
+      <ns0:c r="A2" t="s">
+        <ns0:v>7</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" t="s">
+        <ns0:v>8</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" t="s">
+        <ns0:v>9</ns0:v>
+      </ns0:c>
+      <ns0:c r="D2" t="s">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="E2" t="s">
+        <ns0:v>11</ns0:v>
+      </ns0:c>
+      <ns0:c r="F2">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="G2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" spans="1:7">
+      <ns0:c r="A3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>删除</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" t="s">
+        <ns0:v>13</ns0:v>
+      </ns0:c>
+      <ns0:c r="D3" t="s">
+        <ns0:v>14</ns0:v>
+      </ns0:c>
+      <ns0:c r="E3" t="s">
+        <ns0:v>15</ns0:v>
+      </ns0:c>
+      <ns0:c r="F3">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="G3">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" spans="1:6">
+      <ns0:c r="A4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>删除</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" t="s">
+        <ns0:v>16</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" t="s">
+        <ns0:v>17</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4"/>
+      <ns0:c r="F4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ns0:headerFooter/>
+</ns0:worksheet>
 </file>
</xml_diff>